<commit_message>
08 octubre de 2020 v2
</commit_message>
<xml_diff>
--- a/_downloads/e4b6f84e3db730360c0cc4cfef27c19f/3. Cuenta de Margen Futuros BVC y CME.xlsx
+++ b/_downloads/e4b6f84e3db730360c0cc4cfef27c19f/3. Cuenta de Margen Futuros BVC y CME.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\DERIVADOS FINANCIEROS\CLASES\Futuros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D2802A1-FA41-455A-9028-CD5C4B76B1FA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68823D9C-C28E-4B59-AC33-BD13158D473F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{49894DDF-7A4E-4CA1-B361-16B2C13C2398}"/>
   </bookViews>
@@ -417,11 +417,11 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -754,11 +754,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
     </row>
     <row r="2" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -813,7 +813,7 @@
       </c>
     </row>
     <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="26" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="16"/>
@@ -838,11 +838,11 @@
       <c r="F10" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="20" t="s">
         <v>15</v>
-      </c>
-      <c r="H10" s="21" t="s">
-        <v>16</v>
       </c>
       <c r="L10" s="6"/>
     </row>
@@ -1021,11 +1021,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -1106,7 +1106,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="27" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>